<commit_message>
vault backup: 2026-04-21 21:36:41
</commit_message>
<xml_diff>
--- a/Курсы/Домашняя работа/Домашняя работа 6/Шаблон общей концепции.xlsx
+++ b/Курсы/Домашняя работа/Домашняя работа 6/Шаблон общей концепции.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu\Курсы\Домашняя работа\Домашняя работа 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EF4780-9B2B-4D52-B368-38624B85DBB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{521EA7BB-C23B-4128-8AE2-F524FE3973F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -215,18 +215,6 @@
     </r>
   </si>
   <si>
-    <t>Общая трудоемкость: 108 ак. часов (3 ЗЕТ).
-Контактная работа: 54 часа (лекции + практические занятия в формате «Ты делаешь, я корректирую»).
-Самостоятельная работа: 54 часа.
-Итого: Лекции 23 ч, Практика 31 ч, СРС 54 ч.
-Форматы занятий:
-• Лекции проблемные, с опросами, демонстрацией кода.
-• Практические занятия — полностью в формате «Ты делаешь, я корректирую» (работа в парах/индивидуально, преподаватель ходит и помогает).
-• Каждый модуль завершается тестом (LMS) и домашним заданием (код в Google Colab с автопроверкой части тестов).
-• Итоговый проект — сквозная задача, например: «Предсказание остаточного ресурса подшипника по вибросигналам» или «Классификация брака на конвейере».
-• Экзамен: 30 мин теория (закрытые и открытые вопросы) + 30 мин практика (обучить модель на свежем датасете, предоставляемом во время экзамена).</t>
-  </si>
-  <si>
     <t>Модуль</t>
   </si>
   <si>
@@ -344,12 +332,24 @@
 • Включает нейросетевой эксперимент в свой курсовой или дипломный проект.</t>
     </r>
   </si>
+  <si>
+    <t>Общая трудоемкость: 108 ак. часов (3 ЗЕТ).
+Контактная работа: 54 часа (лекции + практические занятия в формате «Ты делаешь, я корректирую»).
+Самостоятельная работа: 54 часа.
+Итого: Лекции 23 ч, Практика 37 ч, СРС 54 ч.
+Форматы занятий:
+• Лекции проблемные, с опросами, демонстрацией кода.
+• Практические занятия — полностью в формате «Ты делаешь, я корректирую» (работа в парах/индивидуально, преподаватель ходит и помогает).
+• Каждый модуль завершается тестом (LMS) и домашним заданием (код в Google Colab с автопроверкой части тестов).
+• Итоговый проект — сквозная задача, например: «Предсказание остаточного ресурса подшипника по вибросигналам» или «Классификация брака на конвейере».
+• Экзамен: 30 мин теория (закрытые и открытые вопросы) + 30 мин практика (обучить модель на свежем датасете, предоставляемом во время экзамена).</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -391,7 +391,15 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -563,12 +571,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -578,15 +580,21 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -812,29 +820,29 @@
     <col min="2" max="2" width="216.33203125" customWidth="1"/>
     <col min="3" max="26" width="12.6640625" hidden="1"/>
     <col min="28" max="28" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="54.88671875" customWidth="1"/>
-    <col min="33" max="33" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="17.88671875" customWidth="1"/>
+    <col min="30" max="30" width="19.88671875" customWidth="1"/>
+    <col min="31" max="31" width="14.77734375" customWidth="1"/>
+    <col min="32" max="32" width="58.5546875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="22.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
+      <c r="B1" s="6"/>
     </row>
     <row r="2" spans="1:33" ht="42">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:33" ht="122.4">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:33" ht="102">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -842,7 +850,7 @@
       </c>
     </row>
     <row r="4" spans="1:33" ht="224.4">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -850,15 +858,15 @@
       </c>
     </row>
     <row r="5" spans="1:33" ht="266.39999999999998">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>37</v>
+      <c r="B5" s="3" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:33" ht="301.2" customHeight="1">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -866,198 +874,198 @@
       </c>
     </row>
     <row r="7" spans="1:33" ht="334.8" customHeight="1">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:33" ht="306">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:33" ht="285.60000000000002">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:33" ht="13.8">
+      <c r="AB11" s="7" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="11" spans="1:33">
-      <c r="AB11" s="13" t="s">
+      <c r="AC11" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="AC11" s="11" t="s">
+      <c r="AD11" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="AD11" s="11" t="s">
+      <c r="AE11" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="AE11" s="11" t="s">
+      <c r="AF11" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="AF11" s="11" t="s">
+      <c r="AG11" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="AG11" s="12" t="s">
+    </row>
+    <row r="12" spans="1:33" ht="13.8">
+      <c r="AB12" s="10" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:33">
-      <c r="AB12" s="14" t="s">
+      <c r="AC12" s="11">
+        <v>4</v>
+      </c>
+      <c r="AD12" s="11">
+        <v>6</v>
+      </c>
+      <c r="AE12" s="11">
+        <v>8</v>
+      </c>
+      <c r="AF12" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="AC12" s="7">
+      <c r="AG12" s="12">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33" ht="13.8">
+      <c r="AB13" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="AC13" s="11">
+        <v>3</v>
+      </c>
+      <c r="AD13" s="11">
         <v>4</v>
       </c>
-      <c r="AD12" s="7">
+      <c r="AE13" s="11">
         <v>6</v>
       </c>
-      <c r="AE12" s="7">
+      <c r="AF13" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="AG13" s="12">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:33" ht="13.8">
+      <c r="AB14" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="AC14" s="11">
+        <v>4</v>
+      </c>
+      <c r="AD14" s="11">
+        <v>6</v>
+      </c>
+      <c r="AE14" s="11">
         <v>8</v>
       </c>
-      <c r="AF12" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="AG12" s="8">
+      <c r="AF14" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="AG14" s="12">
         <v>0.1</v>
       </c>
     </row>
-    <row r="13" spans="1:33">
-      <c r="AB13" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="AC13" s="7">
+    <row r="15" spans="1:33" ht="13.8">
+      <c r="AB15" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="AC15" s="11">
+        <v>5</v>
+      </c>
+      <c r="AD15" s="11">
+        <v>7</v>
+      </c>
+      <c r="AE15" s="11">
+        <v>12</v>
+      </c>
+      <c r="AF15" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="AG15" s="12">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:33" ht="13.8">
+      <c r="AB16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC16" s="11">
         <v>3</v>
       </c>
-      <c r="AD13" s="7">
+      <c r="AD16" s="11">
+        <v>5</v>
+      </c>
+      <c r="AE16" s="11">
+        <v>8</v>
+      </c>
+      <c r="AF16" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="AG16" s="12">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="17" spans="28:33" ht="13.8">
+      <c r="AB17" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="AC17" s="11">
+        <v>2</v>
+      </c>
+      <c r="AD17" s="11">
+        <v>3</v>
+      </c>
+      <c r="AE17" s="11">
         <v>4</v>
       </c>
-      <c r="AE13" s="7">
+      <c r="AF17" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG17" s="12">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="18" spans="28:33" ht="13.8">
+      <c r="AB18" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC18" s="11">
+        <v>2</v>
+      </c>
+      <c r="AD18" s="11">
         <v>6</v>
       </c>
-      <c r="AF13" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="AG13" s="8">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:33">
-      <c r="AB14" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="AC14" s="7">
-        <v>4</v>
-      </c>
-      <c r="AD14" s="7">
-        <v>6</v>
-      </c>
-      <c r="AE14" s="7">
+      <c r="AE18" s="11">
         <v>8</v>
       </c>
-      <c r="AF14" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="AG14" s="8">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:33">
-      <c r="AB15" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC15" s="7">
-        <v>5</v>
-      </c>
-      <c r="AD15" s="7">
-        <v>7</v>
-      </c>
-      <c r="AE15" s="7">
-        <v>12</v>
-      </c>
-      <c r="AF15" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="AG15" s="8">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:33">
-      <c r="AB16" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="AC16" s="7">
-        <v>3</v>
-      </c>
-      <c r="AD16" s="7">
-        <v>5</v>
-      </c>
-      <c r="AE16" s="7">
-        <v>8</v>
-      </c>
-      <c r="AF16" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="AG16" s="8">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="17" spans="28:33">
-      <c r="AB17" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="AC17" s="7">
-        <v>2</v>
-      </c>
-      <c r="AD17" s="7">
-        <v>3</v>
-      </c>
-      <c r="AE17" s="7">
-        <v>4</v>
-      </c>
-      <c r="AF17" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="AG17" s="8">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="18" spans="28:33">
-      <c r="AB18" s="14" t="s">
+      <c r="AF18" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="AC18" s="7">
-        <v>2</v>
-      </c>
-      <c r="AD18" s="7">
-        <v>6</v>
-      </c>
-      <c r="AE18" s="7">
-        <v>8</v>
-      </c>
-      <c r="AF18" s="7" t="s">
+      <c r="AG18" s="12">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="19" spans="28:33" ht="13.8">
+      <c r="AB19" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="AG18" s="8">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="19" spans="28:33">
-      <c r="AB19" s="15" t="s">
+      <c r="AC19" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="AC19" s="9" t="s">
+      <c r="AD19" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE19" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF19" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="AD19" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE19" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="AF19" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="AG19" s="10">
+      <c r="AG19" s="15">
         <v>0.1</v>
       </c>
     </row>

</xml_diff>